<commit_message>
Update model outputs 2026-08-17 19:17:48
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">Team</t>
   </si>
@@ -35,10 +35,10 @@
     <t xml:space="preserve">Sydney Swans</t>
   </si>
   <si>
-    <t xml:space="preserve">3.39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.91</t>
+    <t xml:space="preserve">3.66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.97</t>
   </si>
   <si>
     <t xml:space="preserve">1.00</t>
@@ -50,121 +50,118 @@
     <t xml:space="preserve">Fremantle</t>
   </si>
   <si>
-    <t xml:space="preserve">3.65</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.97</t>
+    <t xml:space="preserve">3.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.83</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.09</t>
   </si>
   <si>
     <t xml:space="preserve">Brisbane Lions</t>
   </si>
   <si>
-    <t xml:space="preserve">9.29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.07</t>
+    <t xml:space="preserve">9.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.92</t>
   </si>
   <si>
     <t xml:space="preserve">Geelong Cats</t>
   </si>
   <si>
-    <t xml:space="preserve">9.90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.68</t>
-  </si>
-  <si>
-    <t xml:space="preserve">416.67</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.36</t>
+    <t xml:space="preserve">10.19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">303.03</t>
   </si>
   <si>
     <t xml:space="preserve">Adelaide Crows</t>
   </si>
   <si>
-    <t xml:space="preserve">17.67</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.23</t>
+    <t xml:space="preserve">26.60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.61</t>
   </si>
   <si>
     <t xml:space="preserve">Melbourne</t>
   </si>
   <si>
-    <t xml:space="preserve">18.28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.00</t>
+    <t xml:space="preserve">31.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6666.67</t>
   </si>
   <si>
     <t xml:space="preserve">Collingwood</t>
   </si>
   <si>
-    <t xml:space="preserve">90.50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33.67</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2857.14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.53</t>
+    <t xml:space="preserve">141.84</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51.28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1250.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.73</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Western Bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">370.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">135.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.53</t>
   </si>
   <si>
     <t xml:space="preserve">Carlton</t>
   </si>
   <si>
-    <t xml:space="preserve">666.67</t>
-  </si>
-  <si>
-    <t xml:space="preserve">273.97</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13.62</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Western Bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">952.38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">243.90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.71</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.27</t>
+    <t xml:space="preserve">1176.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">317.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.32</t>
   </si>
   <si>
     <t xml:space="preserve">Essendon</t>
@@ -622,41 +619,41 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>24</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s">
         <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>29</v>
-      </c>
-      <c r="D7" t="s">
-        <v>30</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -667,22 +664,22 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
         <v>31</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>32</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>33</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" t="s">
         <v>34</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -742,12 +739,12 @@
         <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -767,7 +764,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
         <v>10</v>
@@ -787,7 +784,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -807,7 +804,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -827,7 +824,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -847,7 +844,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -867,7 +864,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -887,7 +884,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Update model outputs 2026-09-05 08:28:18
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">Team</t>
   </si>
@@ -35,10 +35,10 @@
     <t xml:space="preserve">Sydney Swans</t>
   </si>
   <si>
-    <t xml:space="preserve">3.66</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.97</t>
+    <t xml:space="preserve">4.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16</t>
   </si>
   <si>
     <t xml:space="preserve">1.00</t>
@@ -50,118 +50,79 @@
     <t xml:space="preserve">Fremantle</t>
   </si>
   <si>
-    <t xml:space="preserve">3.68</t>
+    <t xml:space="preserve">4.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brisbane Lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geelong Cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.73</t>
   </si>
   <si>
     <t xml:space="preserve">1.98</t>
   </si>
   <si>
-    <t xml:space="preserve">Hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.83</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisbane Lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geelong Cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">303.03</t>
-  </si>
-  <si>
     <t xml:space="preserve">Adelaide Crows</t>
   </si>
   <si>
-    <t xml:space="preserve">26.60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.61</t>
+    <t xml:space="preserve">25.35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20000.00</t>
   </si>
   <si>
     <t xml:space="preserve">Melbourne</t>
   </si>
   <si>
-    <t xml:space="preserve">31.45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6666.67</t>
+    <t xml:space="preserve">55.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Western Bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carlton</t>
   </si>
   <si>
     <t xml:space="preserve">Collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">141.84</t>
-  </si>
-  <si>
-    <t xml:space="preserve">51.28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1250.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.73</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Western Bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">370.37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">135.14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.53</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1176.47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">317.46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.32</t>
   </si>
   <si>
     <t xml:space="preserve">Essendon</t>
@@ -593,7 +554,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
@@ -604,16 +565,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
@@ -624,36 +585,36 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
       <c r="E6" t="s">
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>27</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -664,87 +625,87 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>31</v>
       </c>
-      <c r="C8" t="s">
-        <v>32</v>
-      </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="F9" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>45</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -764,7 +725,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
         <v>10</v>
@@ -784,7 +745,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -804,7 +765,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -824,7 +785,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -844,7 +805,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -864,7 +825,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -884,7 +845,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Update model outputs 2026-09-09 09:08:16
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">Team</t>
   </si>
@@ -35,10 +35,10 @@
     <t xml:space="preserve">Sydney Swans</t>
   </si>
   <si>
-    <t xml:space="preserve">4.21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16</t>
+    <t xml:space="preserve">3.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.89</t>
   </si>
   <si>
     <t xml:space="preserve">1.00</t>
@@ -50,73 +50,76 @@
     <t xml:space="preserve">Fremantle</t>
   </si>
   <si>
-    <t xml:space="preserve">4.42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.25</t>
+    <t xml:space="preserve">4.79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.30</t>
   </si>
   <si>
     <t xml:space="preserve">Hawthorn</t>
   </si>
   <si>
-    <t xml:space="preserve">5.65</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.68</t>
+    <t xml:space="preserve">6.85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geelong Cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.15</t>
   </si>
   <si>
     <t xml:space="preserve">Brisbane Lions</t>
   </si>
   <si>
-    <t xml:space="preserve">6.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geelong Cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.73</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.98</t>
+    <t xml:space="preserve">7.65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.81</t>
   </si>
   <si>
     <t xml:space="preserve">Adelaide Crows</t>
   </si>
   <si>
-    <t xml:space="preserve">25.35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20000.00</t>
+    <t xml:space="preserve">18.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.31</t>
   </si>
   <si>
     <t xml:space="preserve">Melbourne</t>
   </si>
   <si>
-    <t xml:space="preserve">55.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.86</t>
+    <t xml:space="preserve">60.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.81</t>
   </si>
   <si>
     <t xml:space="preserve">Western Bulldogs</t>
   </si>
   <si>
-    <t xml:space="preserve">99.01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">41.32</t>
+    <t xml:space="preserve">120.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50.25</t>
   </si>
   <si>
     <t xml:space="preserve">Carlton</t>
@@ -554,7 +557,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
@@ -565,16 +568,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
@@ -585,16 +588,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
@@ -605,16 +608,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -625,13 +628,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -645,13 +648,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -665,7 +668,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -685,7 +688,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
@@ -705,7 +708,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -725,7 +728,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
         <v>10</v>
@@ -745,7 +748,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -765,7 +768,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -785,7 +788,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -805,7 +808,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -825,7 +828,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -845,7 +848,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>

</xml_diff>